<commit_message>
add LLD NHNCK Nhóm A
</commit_message>
<xml_diff>
--- a/Source/NHNCK_Source_Tables.xlsx
+++ b/Source/NHNCK_Source_Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc29544db4608b3c/One - UBCK/Design/ubck_atomic_design/Source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_4F676A49A1805012BC8BB73ECD5BEB4AF6CC78B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7E9F568-B7C0-42AD-846A-776682A5755B}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_4F676A49A1805012BC8BB73ECD5BEB4AF6CC78B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B7FCF6A-1514-45C2-9611-A503031300D9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19103" yWindow="-98" windowWidth="22694" windowHeight="14595" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh sách bảng" sheetId="1" r:id="rId1"/>
@@ -4108,7 +4108,7 @@
       <c r="D98" s="2"/>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="4" t="s">
         <v>19</v>
       </c>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="E99" s="4"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="4" t="s">
         <v>19</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="4" t="s">
         <v>19</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="4" t="s">
         <v>43</v>
       </c>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="E181" s="4"/>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="4" t="s">
         <v>43</v>
       </c>
@@ -5298,7 +5298,7 @@
       <c r="D182" s="5"/>
       <c r="E182" s="4"/>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="4" t="s">
         <v>43</v>
       </c>
@@ -5311,7 +5311,7 @@
       <c r="D183" s="5"/>
       <c r="E183" s="4"/>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="4" t="s">
         <v>43</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="4" t="s">
         <v>43</v>
       </c>
@@ -5341,7 +5341,7 @@
       <c r="D185" s="5"/>
       <c r="E185" s="4"/>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="4" t="s">
         <v>43</v>
       </c>
@@ -5354,7 +5354,7 @@
       <c r="D186" s="5"/>
       <c r="E186" s="4"/>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="4" t="s">
         <v>43</v>
       </c>
@@ -7151,7 +7151,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="3" t="s">
         <v>69</v>
       </c>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="E318" s="3"/>
     </row>
-    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="3" t="s">
         <v>69</v>
       </c>
@@ -7179,7 +7179,7 @@
       <c r="D319" s="2"/>
       <c r="E319" s="3"/>
     </row>
-    <row r="320" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="3" t="s">
         <v>69</v>
       </c>
@@ -7192,7 +7192,7 @@
       <c r="D320" s="2"/>
       <c r="E320" s="3"/>
     </row>
-    <row r="321" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="3" t="s">
         <v>69</v>
       </c>
@@ -7205,7 +7205,7 @@
       <c r="D321" s="2"/>
       <c r="E321" s="3"/>
     </row>
-    <row r="322" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="3" t="s">
         <v>69</v>
       </c>
@@ -7218,7 +7218,7 @@
       <c r="D322" s="2"/>
       <c r="E322" s="3"/>
     </row>
-    <row r="323" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="3" t="s">
         <v>69</v>
       </c>
@@ -8519,7 +8519,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="418" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A418" s="3" t="s">
         <v>93</v>
       </c>
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E418" s="3"/>
     </row>
-    <row r="419" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A419" s="3" t="s">
         <v>93</v>
       </c>
@@ -8547,7 +8547,7 @@
       <c r="D419" s="2"/>
       <c r="E419" s="3"/>
     </row>
-    <row r="420" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A420" s="3" t="s">
         <v>93</v>
       </c>
@@ -8560,7 +8560,7 @@
       <c r="D420" s="2"/>
       <c r="E420" s="3"/>
     </row>
-    <row r="421" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A421" s="3" t="s">
         <v>93</v>
       </c>
@@ -8573,7 +8573,7 @@
       <c r="D421" s="2"/>
       <c r="E421" s="3"/>
     </row>
-    <row r="422" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A422" s="3" t="s">
         <v>93</v>
       </c>
@@ -8586,7 +8586,7 @@
       <c r="D422" s="2"/>
       <c r="E422" s="3"/>
     </row>
-    <row r="423" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A423" s="3" t="s">
         <v>93</v>
       </c>
@@ -8599,7 +8599,7 @@
       <c r="D423" s="2"/>
       <c r="E423" s="3"/>
     </row>
-    <row r="424" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A424" s="3" t="s">
         <v>93</v>
       </c>
@@ -8612,7 +8612,7 @@
       <c r="D424" s="2"/>
       <c r="E424" s="3"/>
     </row>
-    <row r="425" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A425" s="3" t="s">
         <v>93</v>
       </c>
@@ -8629,7 +8629,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="426" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A426" s="3" t="s">
         <v>93</v>
       </c>
@@ -8646,7 +8646,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="427" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A427" s="3" t="s">
         <v>93</v>
       </c>
@@ -8663,7 +8663,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="428" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A428" s="3" t="s">
         <v>93</v>
       </c>
@@ -8676,7 +8676,7 @@
       <c r="D428" s="2"/>
       <c r="E428" s="3"/>
     </row>
-    <row r="429" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A429" s="3" t="s">
         <v>93</v>
       </c>
@@ -8689,7 +8689,7 @@
       <c r="D429" s="2"/>
       <c r="E429" s="3"/>
     </row>
-    <row r="430" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A430" s="3" t="s">
         <v>93</v>
       </c>
@@ -8947,8 +8947,8 @@
   <autoFilter ref="A1:E447" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="CertificateDepartments"/>
-        <filter val="Departments"/>
+        <filter val="Positions"/>
+        <filter val="Users"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>